<commit_message>
let S4's labels repel themselves and check panel c survives losing anyone
</commit_message>
<xml_diff>
--- a/04_Figures/S4/c_data/S4.xlsx
+++ b/04_Figures/S4/c_data/S4.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5048" uniqueCount="3078">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5048" uniqueCount="3077">
   <si>
     <t>sheet</t>
   </si>
@@ -8920,15 +8920,6 @@
     <t>cdb8d908fb24ab0d2be6f2d00021db81</t>
   </si>
   <si>
-    <t>helpers</t>
-  </si>
-  <si>
-    <t>02_HRvLR/helpers.R</t>
-  </si>
-  <si>
-    <t>8d6eadd4947a5d7e144163e850427c2a</t>
-  </si>
-  <si>
     <t>01_Processing/05_Set_Scores/c_data/singscore.rds</t>
   </si>
   <si>
@@ -8996,6 +8987,12 @@
   </si>
   <si>
     <t>4.0.3</t>
+  </si>
+  <si>
+    <t>ggrepel</t>
+  </si>
+  <si>
+    <t>0.9.8</t>
   </si>
   <si>
     <t>ggtext</t>
@@ -54893,7 +54890,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -54942,24 +54939,13 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" t="s">
         <v>2966</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>2967</v>
-      </c>
-      <c r="C5" t="s">
-        <v>2968</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>90</v>
-      </c>
-      <c r="B6" t="s">
-        <v>2969</v>
-      </c>
-      <c r="C6" t="s">
-        <v>2970</v>
       </c>
     </row>
   </sheetData>
@@ -54969,7 +54955,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C54"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1">
@@ -54985,585 +54971,596 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>2971</v>
+        <v>2968</v>
       </c>
       <c r="B2" t="s">
-        <v>2972</v>
+        <v>2969</v>
       </c>
       <c r="C2" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>2974</v>
+        <v>2971</v>
       </c>
       <c r="B3" t="s">
-        <v>2975</v>
+        <v>2972</v>
       </c>
       <c r="C3" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>2976</v>
+        <v>2973</v>
       </c>
       <c r="B4" t="s">
-        <v>2977</v>
+        <v>2974</v>
       </c>
       <c r="C4" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>2978</v>
+        <v>2975</v>
       </c>
       <c r="B5" t="s">
-        <v>2979</v>
+        <v>2976</v>
       </c>
       <c r="C5" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>2980</v>
+        <v>2977</v>
       </c>
       <c r="B6" t="s">
-        <v>2981</v>
+        <v>2978</v>
       </c>
       <c r="C6" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>2982</v>
+        <v>2979</v>
       </c>
       <c r="B7" t="s">
-        <v>2983</v>
+        <v>2980</v>
       </c>
       <c r="C7" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>2984</v>
+        <v>2981</v>
       </c>
       <c r="B8" t="s">
-        <v>2985</v>
+        <v>2982</v>
       </c>
       <c r="C8" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>2986</v>
+        <v>2983</v>
       </c>
       <c r="B9" t="s">
-        <v>2987</v>
+        <v>2984</v>
       </c>
       <c r="C9" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>2988</v>
+        <v>2985</v>
       </c>
       <c r="B10" t="s">
-        <v>2989</v>
+        <v>2986</v>
       </c>
       <c r="C10" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>2990</v>
+        <v>2987</v>
       </c>
       <c r="B11" t="s">
-        <v>2991</v>
+        <v>2988</v>
       </c>
       <c r="C11" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>2992</v>
+        <v>2989</v>
       </c>
       <c r="B12" t="s">
-        <v>2993</v>
+        <v>2990</v>
       </c>
       <c r="C12" t="s">
-        <v>2994</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>2995</v>
+        <v>2991</v>
       </c>
       <c r="B13" t="s">
-        <v>2996</v>
+        <v>2992</v>
       </c>
       <c r="C13" t="s">
-        <v>2973</v>
+        <v>2993</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>2997</v>
+        <v>2994</v>
       </c>
       <c r="B14" t="s">
-        <v>2998</v>
+        <v>2995</v>
       </c>
       <c r="C14" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>2999</v>
+        <v>2996</v>
       </c>
       <c r="B15" t="s">
-        <v>3000</v>
+        <v>2997</v>
       </c>
       <c r="C15" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>3001</v>
+        <v>2998</v>
       </c>
       <c r="B16" t="s">
-        <v>3002</v>
+        <v>2999</v>
       </c>
       <c r="C16" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>3003</v>
+        <v>3000</v>
       </c>
       <c r="B17" t="s">
-        <v>3004</v>
+        <v>3001</v>
       </c>
       <c r="C17" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>3005</v>
+        <v>3002</v>
       </c>
       <c r="B18" t="s">
-        <v>3006</v>
+        <v>3003</v>
       </c>
       <c r="C18" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>3007</v>
+        <v>3004</v>
       </c>
       <c r="B19" t="s">
-        <v>3008</v>
+        <v>3005</v>
       </c>
       <c r="C19" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>3009</v>
+        <v>3006</v>
       </c>
       <c r="B20" t="s">
-        <v>3010</v>
+        <v>3007</v>
       </c>
       <c r="C20" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>3011</v>
+        <v>3008</v>
       </c>
       <c r="B21" t="s">
-        <v>3012</v>
+        <v>3009</v>
       </c>
       <c r="C21" t="s">
-        <v>3013</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>3014</v>
+        <v>3010</v>
       </c>
       <c r="B22" t="s">
-        <v>3015</v>
+        <v>3011</v>
       </c>
       <c r="C22" t="s">
-        <v>2994</v>
+        <v>3012</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>3016</v>
+        <v>3013</v>
       </c>
       <c r="B23" t="s">
-        <v>3017</v>
+        <v>3014</v>
       </c>
       <c r="C23" t="s">
-        <v>2973</v>
+        <v>2993</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>3018</v>
+        <v>3015</v>
       </c>
       <c r="B24" t="s">
-        <v>3019</v>
+        <v>3016</v>
       </c>
       <c r="C24" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>3020</v>
+        <v>3017</v>
       </c>
       <c r="B25" t="s">
-        <v>3021</v>
+        <v>3018</v>
       </c>
       <c r="C25" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>3022</v>
+        <v>3019</v>
       </c>
       <c r="B26" t="s">
-        <v>3023</v>
+        <v>3020</v>
       </c>
       <c r="C26" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>3024</v>
+        <v>3021</v>
       </c>
       <c r="B27" t="s">
-        <v>3025</v>
+        <v>3022</v>
       </c>
       <c r="C27" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" t="s">
-        <v>3026</v>
+        <v>3023</v>
       </c>
       <c r="B28" t="s">
-        <v>3027</v>
+        <v>3024</v>
       </c>
       <c r="C28" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" t="s">
-        <v>3028</v>
+        <v>3025</v>
       </c>
       <c r="B29" t="s">
-        <v>3029</v>
+        <v>3026</v>
       </c>
       <c r="C29" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" t="s">
-        <v>3030</v>
+        <v>3027</v>
       </c>
       <c r="B30" t="s">
-        <v>3031</v>
+        <v>3028</v>
       </c>
       <c r="C30" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>3032</v>
+        <v>3029</v>
       </c>
       <c r="B31" t="s">
-        <v>3033</v>
+        <v>3030</v>
       </c>
       <c r="C31" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>3034</v>
+        <v>3031</v>
       </c>
       <c r="B32" t="s">
-        <v>3035</v>
+        <v>3032</v>
       </c>
       <c r="C32" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>3036</v>
+        <v>3033</v>
       </c>
       <c r="B33" t="s">
-        <v>3037</v>
+        <v>3034</v>
       </c>
       <c r="C33" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>3038</v>
+        <v>3035</v>
       </c>
       <c r="B34" t="s">
-        <v>3039</v>
+        <v>3036</v>
       </c>
       <c r="C34" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>3040</v>
+        <v>3037</v>
       </c>
       <c r="B35" t="s">
-        <v>3041</v>
+        <v>3038</v>
       </c>
       <c r="C35" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>3042</v>
+        <v>3039</v>
       </c>
       <c r="B36" t="s">
-        <v>3043</v>
+        <v>3040</v>
       </c>
       <c r="C36" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>3044</v>
+        <v>3041</v>
       </c>
       <c r="B37" t="s">
-        <v>3045</v>
+        <v>3042</v>
       </c>
       <c r="C37" t="s">
-        <v>2994</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>3046</v>
+        <v>3043</v>
       </c>
       <c r="B38" t="s">
-        <v>3047</v>
+        <v>3044</v>
       </c>
       <c r="C38" t="s">
-        <v>2973</v>
+        <v>2993</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>3048</v>
+        <v>3045</v>
       </c>
       <c r="B39" t="s">
-        <v>3049</v>
+        <v>3046</v>
       </c>
       <c r="C39" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>3050</v>
+        <v>3047</v>
       </c>
       <c r="B40" t="s">
-        <v>3051</v>
+        <v>3048</v>
       </c>
       <c r="C40" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>3052</v>
+        <v>3049</v>
       </c>
       <c r="B41" t="s">
-        <v>3053</v>
+        <v>3050</v>
       </c>
       <c r="C41" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>3054</v>
+        <v>3051</v>
       </c>
       <c r="B42" t="s">
-        <v>3055</v>
+        <v>3052</v>
       </c>
       <c r="C42" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>3056</v>
+        <v>3053</v>
       </c>
       <c r="B43" t="s">
-        <v>3057</v>
+        <v>3054</v>
       </c>
       <c r="C43" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>3058</v>
+        <v>3055</v>
       </c>
       <c r="B44" t="s">
-        <v>3059</v>
+        <v>3056</v>
       </c>
       <c r="C44" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>3060</v>
+        <v>3057</v>
       </c>
       <c r="B45" t="s">
-        <v>3061</v>
+        <v>3058</v>
       </c>
       <c r="C45" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>3062</v>
+        <v>3059</v>
       </c>
       <c r="B46" t="s">
-        <v>3027</v>
+        <v>3060</v>
       </c>
       <c r="C46" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>3063</v>
+        <v>3061</v>
       </c>
       <c r="B47" t="s">
-        <v>2985</v>
+        <v>3026</v>
       </c>
       <c r="C47" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>3064</v>
+        <v>3062</v>
       </c>
       <c r="B48" t="s">
-        <v>3065</v>
+        <v>2982</v>
       </c>
       <c r="C48" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>3066</v>
+        <v>3063</v>
       </c>
       <c r="B49" t="s">
-        <v>3067</v>
+        <v>3064</v>
       </c>
       <c r="C49" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>3068</v>
+        <v>3065</v>
       </c>
       <c r="B50" t="s">
-        <v>3069</v>
+        <v>3066</v>
       </c>
       <c r="C50" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>3070</v>
+        <v>3067</v>
       </c>
       <c r="B51" t="s">
-        <v>3071</v>
+        <v>3068</v>
       </c>
       <c r="C51" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>3072</v>
+        <v>3069</v>
       </c>
       <c r="B52" t="s">
-        <v>3073</v>
+        <v>3070</v>
       </c>
       <c r="C52" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>3074</v>
+        <v>3071</v>
       </c>
       <c r="B53" t="s">
-        <v>3075</v>
+        <v>3072</v>
       </c>
       <c r="C53" t="s">
-        <v>2973</v>
+        <v>2970</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
+        <v>3073</v>
+      </c>
+      <c r="B54" t="s">
+        <v>3074</v>
+      </c>
+      <c r="C54" t="s">
+        <v>2970</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" t="s">
+        <v>3075</v>
+      </c>
+      <c r="B55" t="s">
         <v>3076</v>
       </c>
-      <c r="B54" t="s">
-        <v>3077</v>
-      </c>
-      <c r="C54" t="s">
-        <v>2973</v>
+      <c r="C55" t="s">
+        <v>2970</v>
       </c>
     </row>
   </sheetData>

</xml_diff>